<commit_message>
🤖 自動盤後數據、Direct Buy、Swing BuyNow與績效稽核: 2026-08-18 09:58:17
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18T16:25:26+08:00</t>
+          <t>2026-08-18T17:58:13+08:00</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18T16:25:27+08:00</t>
+          <t>2026-08-18T17:58:13+08:00</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18T16:25:26+08:00</t>
+          <t>2026-08-18T17:58:13+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1351,7 +1351,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18T16:25:27+08:00</t>
+          <t>2026-08-18T17:58:13+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-28 06:23:50
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,17 +613,17 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>95.2</v>
+        <v>96.3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>5.43</v>
+        <v>6.64</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>T1-5早期</t>
+          <t>T6-10發展</t>
         </is>
       </c>
       <c r="J2" s="2" t="n"/>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27T14:24:28+08:00</t>
+          <t>2026-08-28T14:23:44+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>958</v>
+        <v>972</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-5.15</v>
+        <v>-3.76</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27T14:24:29+08:00</t>
+          <t>2026-08-28T14:23:45+08:00</t>
         </is>
       </c>
     </row>
@@ -862,21 +862,21 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>95.2</v>
+        <v>96.3</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5.43</v>
+        <v>6.64</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>T1-5早期</t>
+          <t>T6-10發展</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>8.859999999999999</v>
+        <v>15.73</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>-7.2</v>
@@ -900,7 +900,9 @@
       <c r="T2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="U2" s="2" t="n"/>
+      <c r="U2" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
           <t>Tracking</t>
@@ -923,13 +925,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>958</v>
+        <v>972</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-5.15</v>
+        <v>-3.76</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1157,16 +1159,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23564419072</v>
+        <v>23836696576</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.491467</v>
+        <v>32.866894</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.0394945</v>
+        <v>15.213271</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0323298</v>
+        <v>3.0673676</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1221,7 +1223,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27T14:24:28+08:00</t>
+          <t>2026-08-28T14:23:44+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1247,16 +1249,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>458032939008</v>
+        <v>464726556672</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46.52744</v>
+        <v>47.184464</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.083244</v>
+        <v>29.508259</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.7354474</v>
+        <v>4.8046503</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1283,7 +1285,7 @@
         <v>296</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.59</v>
+        <v>20.6</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1311,7 +1313,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27T14:24:29+08:00</t>
+          <t>2026-08-28T14:23:45+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-08-31 06:25:28
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>96.3</v>
+        <v>94.8</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6.64</v>
+        <v>4.98</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28T14:23:44+08:00</t>
+          <t>2026-08-31T14:25:21+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>972</v>
+        <v>912</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-3.76</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28T14:23:45+08:00</t>
+          <t>2026-08-31T14:25:22+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>96.3</v>
+        <v>94.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>6.64</v>
+        <v>4.98</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -925,13 +925,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>972</v>
+        <v>912</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-3.76</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -942,12 +942,14 @@
         <v>2.48</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-8.42</v>
+        <v>-13.37</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-6.04</v>
-      </c>
-      <c r="K3" s="2" t="n"/>
+        <v>-9.699999999999999</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>-9.699999999999999</v>
+      </c>
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
@@ -1159,16 +1161,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23836696576</v>
+        <v>23465408512</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.866894</v>
+        <v>32.35495</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.213271</v>
+        <v>14.976304</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0673676</v>
+        <v>3.0195892</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1223,7 +1225,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28T14:23:44+08:00</t>
+          <t>2026-08-31T14:25:21+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1249,16 +1251,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>464726556672</v>
+        <v>436039712768</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>47.184464</v>
+        <v>44.250362</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.508259</v>
+        <v>27.686762</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.8046503</v>
+        <v>4.508067</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1285,7 +1287,7 @@
         <v>296</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.6</v>
+        <v>20.61</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1313,7 +1315,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28T14:23:45+08:00</t>
+          <t>2026-08-31T14:25:22+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-01 06:23:36
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>94.8</v>
+        <v>95.2</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>4.98</v>
+        <v>5.43</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31T14:25:21+08:00</t>
+          <t>2026-09-01T14:23:30+08:00</t>
         </is>
       </c>
     </row>
@@ -664,17 +664,17 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>912</v>
+        <v>994</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-9.699999999999999</v>
+        <v>-1.58</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>T1-5早期</t>
+          <t>T6-10發展</t>
         </is>
       </c>
       <c r="J3" s="2" t="n"/>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31T14:25:22+08:00</t>
+          <t>2026-09-01T14:23:31+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>94.8</v>
+        <v>95.2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4.98</v>
+        <v>5.43</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -925,17 +925,17 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>912</v>
+        <v>994</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-9.699999999999999</v>
+        <v>-1.58</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>T1-5早期</t>
+          <t>T6-10發展</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -1161,16 +1161,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23465408512</v>
+        <v>23564419072</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.35495</v>
+        <v>32.491467</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.976304</v>
+        <v>15.0394945</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0195892</v>
+        <v>3.0323298</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1225,7 +1225,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31T14:25:21+08:00</t>
+          <t>2026-09-01T14:23:30+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1251,16 +1251,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>436039712768</v>
+        <v>475245051904</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>44.250362</v>
+        <v>48.440544</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27.686762</v>
+        <v>30.176142</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.508067</v>
+        <v>4.913398</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1287,7 +1287,7 @@
         <v>296</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.61</v>
+        <v>20.52</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1315,7 +1315,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31T14:25:22+08:00</t>
+          <t>2026-09-01T14:23:31+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-02 06:24:07
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>95.2</v>
+        <v>92.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>5.43</v>
+        <v>2.44</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01T14:23:30+08:00</t>
+          <t>2026-09-02T14:24:02+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>994</v>
+        <v>967</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-1.58</v>
+        <v>-4.26</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01T14:23:31+08:00</t>
+          <t>2026-09-02T14:24:03+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>95.2</v>
+        <v>92.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5.43</v>
+        <v>2.44</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -925,13 +925,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>994</v>
+        <v>967</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-1.58</v>
+        <v>-4.26</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1161,16 +1161,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23564419072</v>
+        <v>22896099328</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.491467</v>
+        <v>31.569965</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.0394945</v>
+        <v>14.612954</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0323298</v>
+        <v>2.9463289</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1225,7 +1225,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01T14:23:30+08:00</t>
+          <t>2026-09-02T14:24:02+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1251,16 +1251,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>475245051904</v>
+        <v>462335967232</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>48.440544</v>
+        <v>46.987366</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>30.176142</v>
+        <v>29.356468</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.913398</v>
+        <v>4.7799354</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1287,7 +1287,7 @@
         <v>296</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.52</v>
+        <v>20.58</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1315,7 +1315,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01T14:23:31+08:00</t>
+          <t>2026-09-02T14:24:03+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-03 06:23:45
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>92.5</v>
+        <v>91.2</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.44</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02T14:24:02+08:00</t>
+          <t>2026-09-03T14:23:41+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>967</v>
+        <v>927</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-4.26</v>
+        <v>-8.220000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02T14:24:03+08:00</t>
+          <t>2026-09-03T14:23:42+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>92.5</v>
+        <v>91.2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.44</v>
+        <v>1</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -882,12 +882,14 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-4.65</v>
+        <v>-5.59</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
       </c>
-      <c r="L2" s="2" t="n"/>
+      <c r="L2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
@@ -925,13 +927,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>967</v>
+        <v>927</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-4.26</v>
+        <v>-8.220000000000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -990,7 +992,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1161,16 +1163,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22896099328</v>
+        <v>22574315520</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.569965</v>
+        <v>31.126278</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.612954</v>
+        <v>14.407582</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9463289</v>
+        <v>2.904921</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1225,7 +1227,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02T14:24:02+08:00</t>
+          <t>2026-09-03T14:23:41+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1251,16 +1253,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>462335967232</v>
+        <v>443211415552</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46.987366</v>
+        <v>45</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.356468</v>
+        <v>28.142136</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.7799354</v>
+        <v>4.582213</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1287,7 +1289,7 @@
         <v>296</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.58</v>
+        <v>20.6</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1315,7 +1317,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02T14:24:03+08:00</t>
+          <t>2026-09-03T14:23:42+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-04 06:24:29
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,17 +613,17 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>91.2</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1</v>
+        <v>2.88</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>T6-10發展</t>
+          <t>T11-15中段</t>
         </is>
       </c>
       <c r="J2" s="2" t="n"/>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03T14:23:41+08:00</t>
+          <t>2026-09-04T14:24:25+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>927</v>
+        <v>981</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-8.220000000000001</v>
+        <v>-2.87</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03T14:23:42+08:00</t>
+          <t>2026-09-04T14:24:26+08:00</t>
         </is>
       </c>
     </row>
@@ -862,17 +862,17 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>91.2</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1</v>
+        <v>2.88</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>T6-10發展</t>
+          <t>T11-15中段</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -927,13 +927,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>927</v>
+        <v>981</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-8.220000000000001</v>
+        <v>-2.87</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1163,16 +1163,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22574315520</v>
+        <v>22995109888</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.126278</v>
+        <v>31.706484</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.407582</v>
+        <v>14.676146</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.904921</v>
+        <v>2.95907</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1227,7 +1227,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03T14:23:41+08:00</t>
+          <t>2026-09-04T14:24:25+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1253,16 +1253,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>443211415552</v>
+        <v>469029552128</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45</v>
+        <v>47.667637</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>28.142136</v>
+        <v>29.781485</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.582213</v>
+        <v>4.849138</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1289,7 +1289,7 @@
         <v>296</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.6</v>
+        <v>20.58</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1317,7 +1317,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03T14:23:42+08:00</t>
+          <t>2026-09-04T14:24:26+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-07 06:24:55
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.88</v>
+        <v>2.33</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04T14:24:25+08:00</t>
+          <t>2026-09-07T14:24:51+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>981</v>
+        <v>971</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-2.87</v>
+        <v>-3.86</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04T14:24:26+08:00</t>
+          <t>2026-09-07T14:24:51+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.88</v>
+        <v>2.33</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -927,13 +927,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>981</v>
+        <v>971</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-2.87</v>
+        <v>-3.86</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -952,7 +952,9 @@
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
       </c>
-      <c r="L3" s="2" t="n"/>
+      <c r="L3" s="2" t="n">
+        <v>-3.86</v>
+      </c>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="n"/>
@@ -992,7 +994,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1159,44 +1161,44 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22995109888</v>
+        <v>22871347200</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.706484</v>
+        <v>31.535835</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.676146</v>
+        <v>14.597157</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.95907</v>
+        <v>2.9603052</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>31.29</v>
+        <v>29.62</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>8.69</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>3.89</v>
+        <v>3.98</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>0.06</v>
+        <v>15.71</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>-2.61</v>
+        <v>7.89</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>-17.15</v>
+        <v>18.37</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>46.47</v>
+        <v>390.37</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>2.93</v>
@@ -1205,19 +1207,19 @@
         <v>6.33</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>4390420000</v>
+        <v>5080089000</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>1373706000</v>
+        <v>1504950000</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>381503000</v>
+        <v>475622000</v>
       </c>
       <c r="U2" s="2" t="n">
-        <v>170603000</v>
+        <v>201935000</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>0.69769</v>
+        <v>0.82</v>
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
@@ -1227,7 +1229,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04T14:24:25+08:00</t>
+          <t>2026-09-07T14:24:51+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1249,65 +1251,65 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>469029552128</v>
+        <v>464248438784</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>47.667637</v>
+        <v>47.13592</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.781485</v>
+        <v>29.477901</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.849138</v>
+        <v>4.7997074</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>20.83</v>
+        <v>20.64</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>10.55</v>
+        <v>9.35</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>13.56</v>
+        <v>24.84</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>-3.57</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>-14.43</v>
+        <v>-2.44</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>-14.01</v>
+        <v>99.34</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>296</v>
+        <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.58</v>
+        <v>20.6</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>13984798000</v>
+        <v>15214310000</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>2913500000</v>
+        <v>3140439000</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>1475474000</v>
+        <v>1422221000</v>
       </c>
       <c r="U3" s="2" t="n">
-        <v>1895821000</v>
+        <v>3779084000</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>3.96</v>
+        <v>7.9</v>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
@@ -1317,7 +1319,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04T14:24:26+08:00</t>
+          <t>2026-09-07T14:24:51+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-08 06:23:17
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>92.40000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.33</v>
+        <v>-0.78</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T14:24:51+08:00</t>
+          <t>2026-09-08T14:23:12+08:00</t>
         </is>
       </c>
     </row>
@@ -664,17 +664,17 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>971</v>
+        <v>955</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-3.86</v>
+        <v>-5.45</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>T6-10發展</t>
+          <t>T11-15中段</t>
         </is>
       </c>
       <c r="J3" s="2" t="n"/>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T14:24:51+08:00</t>
+          <t>2026-09-08T14:23:13+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>92.40000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.33</v>
+        <v>-0.78</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-5.59</v>
+        <v>-7.25</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -927,17 +927,17 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>971</v>
+        <v>955</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-3.86</v>
+        <v>-5.45</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>T6-10發展</t>
+          <t>T11-15中段</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -1165,16 +1165,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22871347200</v>
+        <v>22178275328</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.535835</v>
+        <v>30.580204</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.597157</v>
+        <v>14.154819</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9603052</v>
+        <v>2.8705988</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1229,7 +1229,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T14:24:51+08:00</t>
+          <t>2026-09-08T14:23:12+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1255,16 +1255,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>464248438784</v>
+        <v>456598618112</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>47.13592</v>
+        <v>46.381737</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.477901</v>
+        <v>28.992168</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.7997074</v>
+        <v>4.7206182</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1291,7 +1291,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.6</v>
+        <v>20.59</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1319,7 +1319,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T14:24:51+08:00</t>
+          <t>2026-09-08T14:23:13+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-10 06:25:41
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>89.59999999999999</v>
+        <v>89.3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.78</v>
+        <v>-1.11</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T14:23:12+08:00</t>
+          <t>2026-09-10T14:25:37+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>955</v>
+        <v>917</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-5.45</v>
+        <v>-9.210000000000001</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T14:23:13+08:00</t>
+          <t>2026-09-10T14:25:38+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>89.59999999999999</v>
+        <v>89.3</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0.78</v>
+        <v>-1.11</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-7.25</v>
+        <v>-7.56</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -890,7 +890,9 @@
       <c r="L2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M2" s="2" t="n"/>
+      <c r="M2" s="2" t="n">
+        <v>-1.11</v>
+      </c>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n"/>
@@ -927,13 +929,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>955</v>
+        <v>917</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-5.45</v>
+        <v>-9.210000000000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1165,16 +1167,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22178275328</v>
+        <v>22104018944</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30.580204</v>
+        <v>30.477816</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.154819</v>
+        <v>14.107426</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.8705988</v>
+        <v>2.8609877</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1229,7 +1231,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T14:23:12+08:00</t>
+          <t>2026-09-10T14:25:37+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1255,16 +1257,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>456598618112</v>
+        <v>438430302208</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46.381737</v>
+        <v>44.66634</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>28.992168</v>
+        <v>27.838552</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.7206182</v>
+        <v>4.5327826</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1291,7 +1293,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.59</v>
+        <v>20.53</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1319,7 +1321,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08T14:23:13+08:00</t>
+          <t>2026-09-10T14:25:38+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-11 06:27:12
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,17 +613,17 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>89.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1.11</v>
+        <v>-4.65</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>T11-15中段</t>
+          <t>T16-20成熟</t>
         </is>
       </c>
       <c r="J2" s="2" t="n"/>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T14:25:37+08:00</t>
+          <t>2026-09-11T14:27:06+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>917</v>
+        <v>902</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-9.210000000000001</v>
+        <v>-10.69</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T14:25:38+08:00</t>
+          <t>2026-09-11T14:27:07+08:00</t>
         </is>
       </c>
     </row>
@@ -862,17 +862,17 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>89.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-1.11</v>
+        <v>-4.65</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>T11-15中段</t>
+          <t>T16-20成熟</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -882,7 +882,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-7.56</v>
+        <v>-10.87</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -929,13 +929,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>917</v>
+        <v>902</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-9.210000000000001</v>
+        <v>-10.69</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         <v>-13.37</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-9.699999999999999</v>
+        <v>-10.69</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1167,16 +1167,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22104018944</v>
+        <v>21311936512</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30.477816</v>
+        <v>29.385664</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.107426</v>
+        <v>13.601895</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.8609877</v>
+        <v>2.758466</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1231,7 +1231,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T14:25:37+08:00</t>
+          <t>2026-09-11T14:27:06+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1257,16 +1257,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>438430302208</v>
+        <v>431258566656</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>44.66634</v>
+        <v>43.91431</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27.838552</v>
+        <v>27.383179</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.5327826</v>
+        <v>4.4586363</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1293,7 +1293,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.53</v>
+        <v>20.54</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1321,7 +1321,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T14:25:38+08:00</t>
+          <t>2026-09-11T14:27:07+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>